<commit_message>
Add Pomerode data and dataset downloads
Process and include Pomerode data in dados.R (new parsing, aggregation, VAR/CT/PRECOS). Persist outputs as CT.rds, VAR_PROD.rds and PRECOS.rds and keep Excel exports. Update app.R to read RDS files, add writexl, a new "Dados" tab with download buttons/handlers (.xlsx and .rds) for CT, VAR_PROD and PRECOS, and minor UI tweaks (color, last-update date, table ordering). Add new raw Excel data files and bump rsconnect bundleId.
</commit_message>
<xml_diff>
--- a/CT.xlsx
+++ b/CT.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F164"/>
+  <dimension ref="A1:F173"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="6" max="6" width="20.7109375" style="2" customWidth="1"/>
@@ -2235,6 +2235,9 @@
           <t>Agosto</t>
         </is>
       </c>
+      <c r="D78">
+        <v>594.73</v>
+      </c>
       <c r="F78" s="2">
         <v>46235</v>
       </c>
@@ -3287,6 +3290,12 @@
           <t>Setembro</t>
         </is>
       </c>
+      <c r="D128">
+        <v>674.26</v>
+      </c>
+      <c r="E128">
+        <v>8.220000000000001</v>
+      </c>
       <c r="F128" s="2">
         <v>46266</v>
       </c>
@@ -4035,6 +4044,195 @@
         <v>7.04</v>
       </c>
       <c r="F164" s="2">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Janeiro</t>
+        </is>
+      </c>
+      <c r="F165" s="2">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Fevereiro</t>
+        </is>
+      </c>
+      <c r="F166" s="2">
+        <v>46054</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Março</t>
+        </is>
+      </c>
+      <c r="F167" s="2">
+        <v>46082</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="F168" s="2">
+        <v>46113</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Maio</t>
+        </is>
+      </c>
+      <c r="F169" s="2">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Junho</t>
+        </is>
+      </c>
+      <c r="F170" s="2">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Julho</t>
+        </is>
+      </c>
+      <c r="F171" s="2">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="D172">
+        <v>705.25</v>
+      </c>
+      <c r="F172" s="2">
+        <v>46235</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Setembro</t>
+        </is>
+      </c>
+      <c r="D173">
+        <v>751.7</v>
+      </c>
+      <c r="E173">
+        <v>6.59</v>
+      </c>
+      <c r="F173" s="2">
         <v>46266</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor data pipeline and app config
This commit generalizes the data ingestion pipeline in `dados.R` to process every city from `data/` with a shared workflow, avoids locale-dependent month parsing, and keeps the exported CT/VAR_PROD/PRECOS datasets consistent. It also updates `app.R` to centralize project metadata, compute the last update dynamically, and render month labels without relying on a system locale. The changeset adds the new Massaranduba 2026 spreadsheet files, refreshes deployment metadata, and removes obsolete app variants and the visit counter database.
</commit_message>
<xml_diff>
--- a/CT.xlsx
+++ b/CT.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F173"/>
+  <dimension ref="A1:F172"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="6" max="6" width="20.7109375" style="2" customWidth="1"/>
@@ -2439,7 +2439,7 @@
         </is>
       </c>
       <c r="D88">
-        <v>648.5700000000001</v>
+        <v>632.52</v>
       </c>
       <c r="F88" s="2">
         <v>45901</v>
@@ -2465,7 +2465,7 @@
         <v>648.67</v>
       </c>
       <c r="E89">
-        <v>0.02</v>
+        <v>2.55</v>
       </c>
       <c r="F89" s="2">
         <v>45931</v>
@@ -2525,11 +2525,16 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="D92">
-        <v>616.47</v>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Janeiro</t>
+        </is>
+      </c>
+      <c r="F92" s="2">
+        <v>46023</v>
       </c>
     </row>
     <row r="93">
@@ -2545,11 +2550,11 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F93" s="2">
-        <v>46023</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="94">
@@ -2565,11 +2570,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="F94" s="2">
-        <v>46054</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="95">
@@ -2585,11 +2590,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="F95" s="2">
-        <v>46082</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="96">
@@ -2605,11 +2610,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F96" s="2">
-        <v>46113</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="97">
@@ -2625,11 +2630,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F97" s="2">
-        <v>46143</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="98">
@@ -2645,11 +2650,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F98" s="2">
-        <v>46174</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="99">
@@ -2665,11 +2670,14 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Julho</t>
-        </is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="D99">
+        <v>700.12</v>
       </c>
       <c r="F99" s="2">
-        <v>46204</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="100">
@@ -2685,20 +2693,23 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="D100">
-        <v>700.12</v>
+        <v>697.37</v>
+      </c>
+      <c r="E100">
+        <v>-0.39</v>
       </c>
       <c r="F100" s="2">
-        <v>46235</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Brusque</t>
+          <t>Bombinhas</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2708,17 +2719,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Setembro</t>
-        </is>
-      </c>
-      <c r="D101">
-        <v>697.37</v>
-      </c>
-      <c r="E101">
-        <v>-0.39</v>
+          <t>Janeiro</t>
+        </is>
       </c>
       <c r="F101" s="2">
-        <v>46266</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="102">
@@ -2734,11 +2739,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F102" s="2">
-        <v>46023</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="103">
@@ -2754,11 +2759,14 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
-        </is>
+          <t>Março</t>
+        </is>
+      </c>
+      <c r="D103">
+        <v>671.45</v>
       </c>
       <c r="F103" s="2">
-        <v>46054</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="104">
@@ -2774,14 +2782,17 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="D104">
-        <v>671.45</v>
+        <v>702.71</v>
+      </c>
+      <c r="E104">
+        <v>4.66</v>
       </c>
       <c r="F104" s="2">
-        <v>46082</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="105">
@@ -2797,17 +2808,17 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="D105">
-        <v>702.71</v>
+        <v>760.8099999999999</v>
       </c>
       <c r="E105">
-        <v>4.66</v>
+        <v>8.27</v>
       </c>
       <c r="F105" s="2">
-        <v>46113</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="106">
@@ -2823,17 +2834,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Maio</t>
-        </is>
-      </c>
-      <c r="D106">
-        <v>760.8099999999999</v>
-      </c>
-      <c r="E106">
-        <v>8.27</v>
+          <t>Junho</t>
+        </is>
       </c>
       <c r="F106" s="2">
-        <v>46143</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="107">
@@ -2849,11 +2854,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F107" s="2">
-        <v>46174</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="108">
@@ -2869,11 +2874,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="F108" s="2">
-        <v>46204</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="109">
@@ -2889,17 +2894,17 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="F109" s="2">
-        <v>46235</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Bombinhas</t>
+          <t>Indaial</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -2909,11 +2914,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F110" s="2">
-        <v>46266</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="111">
@@ -2929,11 +2934,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F111" s="2">
-        <v>46023</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="112">
@@ -2949,11 +2954,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="F112" s="2">
-        <v>46054</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="113">
@@ -2969,11 +2974,14 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Março</t>
-        </is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="D113">
+        <v>702.88</v>
       </c>
       <c r="F113" s="2">
-        <v>46082</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="114">
@@ -2989,14 +2997,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="D114">
-        <v>702.88</v>
+          <t>Maio</t>
+        </is>
       </c>
       <c r="F114" s="2">
-        <v>46113</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="115">
@@ -3012,11 +3017,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F115" s="2">
-        <v>46143</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="116">
@@ -3032,11 +3037,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F116" s="2">
-        <v>46174</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="117">
@@ -3052,11 +3057,14 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Julho</t>
-        </is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="D117">
+        <v>610.3</v>
       </c>
       <c r="F117" s="2">
-        <v>46204</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="118">
@@ -3072,20 +3080,17 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="D118">
-        <v>610.3</v>
+          <t>Setembro</t>
+        </is>
       </c>
       <c r="F118" s="2">
-        <v>46235</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Indaial</t>
+          <t>Jaraguá do Sul</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3095,11 +3100,11 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F119" s="2">
-        <v>46266</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="120">
@@ -3115,11 +3120,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F120" s="2">
-        <v>46023</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="121">
@@ -3135,11 +3140,14 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
-        </is>
+          <t>Março</t>
+        </is>
+      </c>
+      <c r="D121">
+        <v>642.83</v>
       </c>
       <c r="F121" s="2">
-        <v>46054</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="122">
@@ -3155,14 +3163,17 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="D122">
-        <v>642.83</v>
+        <v>723.75</v>
+      </c>
+      <c r="E122">
+        <v>12.59</v>
       </c>
       <c r="F122" s="2">
-        <v>46082</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="123">
@@ -3178,17 +3189,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="D123">
-        <v>723.75</v>
-      </c>
-      <c r="E123">
-        <v>12.59</v>
+          <t>Maio</t>
+        </is>
       </c>
       <c r="F123" s="2">
-        <v>46113</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="124">
@@ -3204,11 +3209,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F124" s="2">
-        <v>46143</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="125">
@@ -3224,11 +3229,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F125" s="2">
-        <v>46174</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="126">
@@ -3244,11 +3249,14 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Julho</t>
-        </is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="D126">
+        <v>623.02</v>
       </c>
       <c r="F126" s="2">
-        <v>46204</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="127">
@@ -3264,20 +3272,23 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="D127">
-        <v>623.02</v>
+        <v>674.26</v>
+      </c>
+      <c r="E127">
+        <v>8.220000000000001</v>
       </c>
       <c r="F127" s="2">
-        <v>46235</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Jaraguá do Sul</t>
+          <t>Massaranduba</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3287,17 +3298,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Setembro</t>
-        </is>
-      </c>
-      <c r="D128">
-        <v>674.26</v>
-      </c>
-      <c r="E128">
-        <v>8.220000000000001</v>
+          <t>Janeiro</t>
+        </is>
       </c>
       <c r="F128" s="2">
-        <v>46266</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="129">
@@ -3313,11 +3318,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F129" s="2">
-        <v>46023</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="130">
@@ -3333,11 +3338,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="F130" s="2">
-        <v>46054</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="131">
@@ -3353,11 +3358,14 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Março</t>
-        </is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="D131">
+        <v>593.53</v>
       </c>
       <c r="F131" s="2">
-        <v>46082</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="132">
@@ -3373,14 +3381,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="D132">
-        <v>593.53</v>
+          <t>Maio</t>
+        </is>
       </c>
       <c r="F132" s="2">
-        <v>46113</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="133">
@@ -3396,11 +3401,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F133" s="2">
-        <v>46143</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="134">
@@ -3416,11 +3421,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F134" s="2">
-        <v>46174</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="135">
@@ -3436,11 +3441,14 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Julho</t>
-        </is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="D135">
+        <v>653.8</v>
       </c>
       <c r="F135" s="2">
-        <v>46204</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="136">
@@ -3456,17 +3464,23 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
+          <t>Setembro</t>
+        </is>
+      </c>
+      <c r="D136">
+        <v>694.64</v>
+      </c>
+      <c r="E136">
+        <v>6.25</v>
       </c>
       <c r="F136" s="2">
-        <v>46235</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Massaranduba</t>
+          <t>Navegantes</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3476,11 +3490,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F137" s="2">
-        <v>46266</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="138">
@@ -3496,11 +3510,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F138" s="2">
-        <v>46023</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="139">
@@ -3516,11 +3530,11 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="F139" s="2">
-        <v>46054</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="140">
@@ -3536,11 +3550,14 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Março</t>
-        </is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="D140">
+        <v>684.72</v>
       </c>
       <c r="F140" s="2">
-        <v>46082</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="141">
@@ -3556,14 +3573,11 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="D141">
-        <v>684.72</v>
+          <t>Maio</t>
+        </is>
       </c>
       <c r="F141" s="2">
-        <v>46113</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="142">
@@ -3579,11 +3593,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F142" s="2">
-        <v>46143</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="143">
@@ -3599,11 +3613,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F143" s="2">
-        <v>46174</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="144">
@@ -3619,11 +3633,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="F144" s="2">
-        <v>46204</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="145">
@@ -3639,17 +3653,17 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="F145" s="2">
-        <v>46235</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Navegantes</t>
+          <t>Timbó</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3659,11 +3673,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F146" s="2">
-        <v>46266</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="147">
@@ -3679,11 +3693,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F147" s="2">
-        <v>46023</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="148">
@@ -3699,11 +3713,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="F148" s="2">
-        <v>46054</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="149">
@@ -3719,11 +3733,14 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Março</t>
-        </is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="D149">
+        <v>760.12</v>
       </c>
       <c r="F149" s="2">
-        <v>46082</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="150">
@@ -3739,14 +3756,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="D150">
-        <v>760.12</v>
+          <t>Maio</t>
+        </is>
       </c>
       <c r="F150" s="2">
-        <v>46113</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="151">
@@ -3762,11 +3776,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F151" s="2">
-        <v>46143</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="152">
@@ -3782,11 +3796,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F152" s="2">
-        <v>46174</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="153">
@@ -3802,11 +3816,14 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Julho</t>
-        </is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="D153">
+        <v>650.8200000000001</v>
       </c>
       <c r="F153" s="2">
-        <v>46204</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="154">
@@ -3822,20 +3839,23 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="D154">
-        <v>650.8200000000001</v>
+        <v>641.26</v>
+      </c>
+      <c r="E154">
+        <v>-1.47</v>
       </c>
       <c r="F154" s="2">
-        <v>46235</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Timbó</t>
+          <t>Balneário Camboriú</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -3845,17 +3865,11 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Setembro</t>
-        </is>
-      </c>
-      <c r="D155">
-        <v>641.26</v>
-      </c>
-      <c r="E155">
-        <v>-1.47</v>
+          <t>Janeiro</t>
+        </is>
       </c>
       <c r="F155" s="2">
-        <v>46266</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="156">
@@ -3871,11 +3885,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F156" s="2">
-        <v>46023</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="157">
@@ -3891,11 +3905,11 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="F157" s="2">
-        <v>46054</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="158">
@@ -3911,11 +3925,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="F158" s="2">
-        <v>46082</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="159">
@@ -3931,11 +3945,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F159" s="2">
-        <v>46113</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="160">
@@ -3951,11 +3965,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F160" s="2">
-        <v>46143</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="161">
@@ -3971,11 +3985,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F161" s="2">
-        <v>46174</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="162">
@@ -3991,11 +4005,14 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Julho</t>
-        </is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="D162">
+        <v>689.67</v>
       </c>
       <c r="F162" s="2">
-        <v>46204</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="163">
@@ -4011,20 +4028,23 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="D163">
-        <v>689.67</v>
+        <v>738.25</v>
+      </c>
+      <c r="E163">
+        <v>7.04</v>
       </c>
       <c r="F163" s="2">
-        <v>46235</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Balneário Camboriú</t>
+          <t>Pomerode</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -4034,17 +4054,11 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Setembro</t>
-        </is>
-      </c>
-      <c r="D164">
-        <v>738.25</v>
-      </c>
-      <c r="E164">
-        <v>7.04</v>
+          <t>Janeiro</t>
+        </is>
       </c>
       <c r="F164" s="2">
-        <v>46266</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="165">
@@ -4060,11 +4074,11 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F165" s="2">
-        <v>46023</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="166">
@@ -4080,11 +4094,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="F166" s="2">
-        <v>46054</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="167">
@@ -4100,11 +4114,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="F167" s="2">
-        <v>46082</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="168">
@@ -4120,11 +4134,11 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F168" s="2">
-        <v>46113</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="169">
@@ -4140,11 +4154,11 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F169" s="2">
-        <v>46143</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="170">
@@ -4160,11 +4174,11 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F170" s="2">
-        <v>46174</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="171">
@@ -4180,11 +4194,14 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Julho</t>
-        </is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="D171">
+        <v>705.25</v>
       </c>
       <c r="F171" s="2">
-        <v>46204</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="172">
@@ -4200,39 +4217,16 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="D172">
-        <v>705.25</v>
+        <v>751.7</v>
+      </c>
+      <c r="E172">
+        <v>6.59</v>
       </c>
       <c r="F172" s="2">
-        <v>46235</v>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>Pomerode</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>Setembro</t>
-        </is>
-      </c>
-      <c r="D173">
-        <v>751.7</v>
-      </c>
-      <c r="E173">
-        <v>6.59</v>
-      </c>
-      <c r="F173" s="2">
         <v>46266</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh market data for October 2026
This commit adds the latest October 2026 Excel files for Balneário, Brusque, Indaial, Jaraguá, and Timbó, updates the generated CT/PRECOS/VAR_PROD data artifacts, and refreshes the local R session metadata. It also redeploys the Shiny app to shinyapps.io with the latest bundle so the dashboard reflects the updated pricing dataset.
</commit_message>
<xml_diff>
--- a/CT.xlsx
+++ b/CT.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F173"/>
+  <dimension ref="A1:F186"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="6" max="6" width="20.7109375" style="2" customWidth="1"/>
@@ -1506,21 +1506,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Gaspar</t>
+          <t>Blumenau</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Outubro</t>
         </is>
       </c>
       <c r="F47" s="2">
-        <v>45292</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="48">
@@ -1536,14 +1536,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
-        </is>
-      </c>
-      <c r="D48">
-        <v>607.9</v>
+          <t>Janeiro</t>
+        </is>
       </c>
       <c r="F48" s="2">
-        <v>45323</v>
+        <v>45292</v>
       </c>
     </row>
     <row r="49">
@@ -1559,17 +1556,14 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="D49">
-        <v>635.98</v>
-      </c>
-      <c r="E49">
-        <v>4.62</v>
+        <v>607.9</v>
       </c>
       <c r="F49" s="2">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="50">
@@ -1585,17 +1579,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="D50">
-        <v>619.6900000000001</v>
+        <v>635.98</v>
       </c>
       <c r="E50">
-        <v>-2.56</v>
+        <v>4.62</v>
       </c>
       <c r="F50" s="2">
-        <v>45383</v>
+        <v>45352</v>
       </c>
     </row>
     <row r="51">
@@ -1611,17 +1605,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="D51">
-        <v>609.0599999999999</v>
+        <v>619.6900000000001</v>
       </c>
       <c r="E51">
-        <v>-1.71</v>
+        <v>-2.56</v>
       </c>
       <c r="F51" s="2">
-        <v>45413</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="52">
@@ -1637,17 +1631,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="D52">
-        <v>629.77</v>
+        <v>609.0599999999999</v>
       </c>
       <c r="E52">
-        <v>3.4</v>
+        <v>-1.71</v>
       </c>
       <c r="F52" s="2">
-        <v>45444</v>
+        <v>45413</v>
       </c>
     </row>
     <row r="53">
@@ -1663,17 +1657,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="D53">
-        <v>584.47</v>
+        <v>629.77</v>
       </c>
       <c r="E53">
-        <v>-7.19</v>
+        <v>3.4</v>
       </c>
       <c r="F53" s="2">
-        <v>45474</v>
+        <v>45444</v>
       </c>
     </row>
     <row r="54">
@@ -1689,17 +1683,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="D54">
-        <v>579.48</v>
+        <v>584.47</v>
       </c>
       <c r="E54">
-        <v>-0.85</v>
+        <v>-7.19</v>
       </c>
       <c r="F54" s="2">
-        <v>45505</v>
+        <v>45474</v>
       </c>
     </row>
     <row r="55">
@@ -1715,17 +1709,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="D55">
-        <v>568.58</v>
+        <v>579.48</v>
       </c>
       <c r="E55">
-        <v>-1.88</v>
+        <v>-0.85</v>
       </c>
       <c r="F55" s="2">
-        <v>45536</v>
+        <v>45505</v>
       </c>
     </row>
     <row r="56">
@@ -1741,17 +1735,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Outubro</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="D56">
-        <v>554.67</v>
+        <v>568.58</v>
       </c>
       <c r="E56">
-        <v>-2.45</v>
+        <v>-1.88</v>
       </c>
       <c r="F56" s="2">
-        <v>45566</v>
+        <v>45536</v>
       </c>
     </row>
     <row r="57">
@@ -1767,17 +1761,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Novembro</t>
+          <t>Outubro</t>
         </is>
       </c>
       <c r="D57">
-        <v>591.6</v>
+        <v>554.67</v>
       </c>
       <c r="E57">
-        <v>6.66</v>
+        <v>-2.45</v>
       </c>
       <c r="F57" s="2">
-        <v>45597</v>
+        <v>45566</v>
       </c>
     </row>
     <row r="58">
@@ -1793,17 +1787,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Dezembro</t>
+          <t>Novembro</t>
         </is>
       </c>
       <c r="D58">
-        <v>565.35</v>
+        <v>591.6</v>
       </c>
       <c r="E58">
-        <v>-4.44</v>
+        <v>6.66</v>
       </c>
       <c r="F58" s="2">
-        <v>45627</v>
+        <v>45597</v>
       </c>
     </row>
     <row r="59">
@@ -1814,22 +1808,22 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Dezembro</t>
         </is>
       </c>
       <c r="D59">
-        <v>584.49</v>
+        <v>565.35</v>
       </c>
       <c r="E59">
-        <v>3.39</v>
+        <v>-4.44</v>
       </c>
       <c r="F59" s="2">
-        <v>45658</v>
+        <v>45627</v>
       </c>
     </row>
     <row r="60">
@@ -1845,17 +1839,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="D60">
-        <v>617.45</v>
+        <v>584.49</v>
       </c>
       <c r="E60">
-        <v>5.64</v>
+        <v>3.39</v>
       </c>
       <c r="F60" s="2">
-        <v>45689</v>
+        <v>45658</v>
       </c>
     </row>
     <row r="61">
@@ -1871,17 +1865,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="D61">
-        <v>618.61</v>
+        <v>617.45</v>
       </c>
       <c r="E61">
-        <v>0.19</v>
+        <v>5.64</v>
       </c>
       <c r="F61" s="2">
-        <v>45717</v>
+        <v>45689</v>
       </c>
     </row>
     <row r="62">
@@ -1897,11 +1891,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Abril</t>
-        </is>
+          <t>Março</t>
+        </is>
+      </c>
+      <c r="D62">
+        <v>618.61</v>
+      </c>
+      <c r="E62">
+        <v>0.19</v>
       </c>
       <c r="F62" s="2">
-        <v>45748</v>
+        <v>45717</v>
       </c>
     </row>
     <row r="63">
@@ -1917,11 +1917,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="F63" s="2">
-        <v>45778</v>
+        <v>45748</v>
       </c>
     </row>
     <row r="64">
@@ -1937,11 +1937,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F64" s="2">
-        <v>45809</v>
+        <v>45778</v>
       </c>
     </row>
     <row r="65">
@@ -1957,11 +1957,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F65" s="2">
-        <v>45839</v>
+        <v>45809</v>
       </c>
     </row>
     <row r="66">
@@ -1977,11 +1977,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F66" s="2">
-        <v>45870</v>
+        <v>45839</v>
       </c>
     </row>
     <row r="67">
@@ -1997,11 +1997,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="F67" s="2">
-        <v>45901</v>
+        <v>45870</v>
       </c>
     </row>
     <row r="68">
@@ -2017,11 +2017,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Outubro</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="F68" s="2">
-        <v>45931</v>
+        <v>45901</v>
       </c>
     </row>
     <row r="69">
@@ -2037,11 +2037,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Novembro</t>
+          <t>Outubro</t>
         </is>
       </c>
       <c r="F69" s="2">
-        <v>45962</v>
+        <v>45931</v>
       </c>
     </row>
     <row r="70">
@@ -2057,11 +2057,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Dezembro</t>
+          <t>Novembro</t>
         </is>
       </c>
       <c r="F70" s="2">
-        <v>45992</v>
+        <v>45962</v>
       </c>
     </row>
     <row r="71">
@@ -2072,16 +2072,16 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Dezembro</t>
         </is>
       </c>
       <c r="F71" s="2">
-        <v>46023</v>
+        <v>45992</v>
       </c>
     </row>
     <row r="72">
@@ -2097,11 +2097,11 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F72" s="2">
-        <v>46054</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="73">
@@ -2117,14 +2117,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Março</t>
-        </is>
-      </c>
-      <c r="D73">
-        <v>584.04</v>
+          <t>Fevereiro</t>
+        </is>
       </c>
       <c r="F73" s="2">
-        <v>46082</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="74">
@@ -2140,17 +2137,14 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="D74">
-        <v>618.51</v>
-      </c>
-      <c r="E74">
-        <v>5.9</v>
+        <v>584.04</v>
       </c>
       <c r="F74" s="2">
-        <v>46113</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="75">
@@ -2166,17 +2160,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="D75">
-        <v>648.72</v>
+        <v>618.51</v>
       </c>
       <c r="E75">
-        <v>4.88</v>
+        <v>5.9</v>
       </c>
       <c r="F75" s="2">
-        <v>46143</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="76">
@@ -2192,11 +2186,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Junho</t>
-        </is>
+          <t>Maio</t>
+        </is>
+      </c>
+      <c r="D76">
+        <v>648.72</v>
+      </c>
+      <c r="E76">
+        <v>4.88</v>
       </c>
       <c r="F76" s="2">
-        <v>46174</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="77">
@@ -2212,11 +2212,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F77" s="2">
-        <v>46204</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="78">
@@ -2232,14 +2232,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="D78">
-        <v>594.73</v>
+          <t>Julho</t>
+        </is>
       </c>
       <c r="F78" s="2">
-        <v>46235</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="79">
@@ -2255,57 +2252,60 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="D79">
-        <v>624.9400000000001</v>
-      </c>
-      <c r="E79">
-        <v>5.08</v>
+        <v>594.73</v>
       </c>
       <c r="F79" s="2">
-        <v>46266</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Brusque</t>
+          <t>Gaspar</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Janeiro</t>
-        </is>
+          <t>Setembro</t>
+        </is>
+      </c>
+      <c r="D80">
+        <v>624.9400000000001</v>
+      </c>
+      <c r="E80">
+        <v>5.08</v>
       </c>
       <c r="F80" s="2">
-        <v>45658</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Brusque</t>
+          <t>Gaspar</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Outubro</t>
         </is>
       </c>
       <c r="F81" s="2">
-        <v>45689</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="82">
@@ -2321,11 +2321,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F82" s="2">
-        <v>45717</v>
+        <v>45658</v>
       </c>
     </row>
     <row r="83">
@@ -2341,11 +2341,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F83" s="2">
-        <v>45748</v>
+        <v>45689</v>
       </c>
     </row>
     <row r="84">
@@ -2361,11 +2361,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="F84" s="2">
-        <v>45778</v>
+        <v>45717</v>
       </c>
     </row>
     <row r="85">
@@ -2381,11 +2381,11 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="F85" s="2">
-        <v>45809</v>
+        <v>45748</v>
       </c>
     </row>
     <row r="86">
@@ -2401,11 +2401,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F86" s="2">
-        <v>45839</v>
+        <v>45778</v>
       </c>
     </row>
     <row r="87">
@@ -2421,11 +2421,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F87" s="2">
-        <v>45870</v>
+        <v>45809</v>
       </c>
     </row>
     <row r="88">
@@ -2441,14 +2441,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Setembro</t>
-        </is>
-      </c>
-      <c r="D88">
-        <v>632.52</v>
+          <t>Julho</t>
+        </is>
       </c>
       <c r="F88" s="2">
-        <v>45901</v>
+        <v>45839</v>
       </c>
     </row>
     <row r="89">
@@ -2464,17 +2461,11 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Outubro</t>
-        </is>
-      </c>
-      <c r="D89">
-        <v>648.67</v>
-      </c>
-      <c r="E89">
-        <v>2.55</v>
+          <t>Agosto</t>
+        </is>
       </c>
       <c r="F89" s="2">
-        <v>45931</v>
+        <v>45870</v>
       </c>
     </row>
     <row r="90">
@@ -2490,17 +2481,14 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Novembro</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="D90">
-        <v>625.33</v>
-      </c>
-      <c r="E90">
-        <v>-3.6</v>
+        <v>632.52</v>
       </c>
       <c r="F90" s="2">
-        <v>45962</v>
+        <v>45901</v>
       </c>
     </row>
     <row r="91">
@@ -2516,11 +2504,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Dezembro</t>
-        </is>
+          <t>Outubro</t>
+        </is>
+      </c>
+      <c r="D91">
+        <v>648.67</v>
+      </c>
+      <c r="E91">
+        <v>2.55</v>
       </c>
       <c r="F91" s="2">
-        <v>45992</v>
+        <v>45931</v>
       </c>
     </row>
     <row r="92">
@@ -2531,16 +2525,22 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Janeiro</t>
-        </is>
+          <t>Novembro</t>
+        </is>
+      </c>
+      <c r="D92">
+        <v>625.33</v>
+      </c>
+      <c r="E92">
+        <v>-3.6</v>
       </c>
       <c r="F92" s="2">
-        <v>46023</v>
+        <v>45962</v>
       </c>
     </row>
     <row r="93">
@@ -2551,16 +2551,16 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Dezembro</t>
         </is>
       </c>
       <c r="F93" s="2">
-        <v>46054</v>
+        <v>45992</v>
       </c>
     </row>
     <row r="94">
@@ -2576,11 +2576,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F94" s="2">
-        <v>46082</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="95">
@@ -2596,11 +2596,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F95" s="2">
-        <v>46113</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="96">
@@ -2616,11 +2616,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="F96" s="2">
-        <v>46143</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="97">
@@ -2636,11 +2636,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="F97" s="2">
-        <v>46174</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="98">
@@ -2656,11 +2656,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F98" s="2">
-        <v>46204</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="99">
@@ -2676,14 +2676,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="D99">
-        <v>700.12</v>
+          <t>Junho</t>
+        </is>
       </c>
       <c r="F99" s="2">
-        <v>46235</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="100">
@@ -2699,23 +2696,17 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Setembro</t>
-        </is>
-      </c>
-      <c r="D100">
-        <v>697.37</v>
-      </c>
-      <c r="E100">
-        <v>-0.39</v>
+          <t>Julho</t>
+        </is>
       </c>
       <c r="F100" s="2">
-        <v>46266</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Bombinhas</t>
+          <t>Brusque</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2725,17 +2716,20 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Janeiro</t>
-        </is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="D101">
+        <v>700.12</v>
       </c>
       <c r="F101" s="2">
-        <v>46023</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Bombinhas</t>
+          <t>Brusque</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2745,17 +2739,23 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
-        </is>
+          <t>Setembro</t>
+        </is>
+      </c>
+      <c r="D102">
+        <v>697.37</v>
+      </c>
+      <c r="E102">
+        <v>-0.39</v>
       </c>
       <c r="F102" s="2">
-        <v>46054</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Bombinhas</t>
+          <t>Brusque</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2765,20 +2765,23 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Outubro</t>
         </is>
       </c>
       <c r="D103">
-        <v>671.45</v>
+        <v>762.29</v>
+      </c>
+      <c r="E103">
+        <v>9.31</v>
       </c>
       <c r="F103" s="2">
-        <v>46082</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Bombinhas</t>
+          <t>Brusque</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2786,19 +2789,11 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>Abril</t>
-        </is>
-      </c>
       <c r="D104">
-        <v>702.71</v>
+        <v>682.34</v>
       </c>
       <c r="E104">
-        <v>4.66</v>
-      </c>
-      <c r="F104" s="2">
-        <v>46113</v>
+        <v>-10.49</v>
       </c>
     </row>
     <row r="105">
@@ -2814,17 +2809,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Maio</t>
-        </is>
-      </c>
-      <c r="D105">
-        <v>760.8099999999999</v>
-      </c>
-      <c r="E105">
-        <v>8.27</v>
+          <t>Janeiro</t>
+        </is>
       </c>
       <c r="F105" s="2">
-        <v>46143</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="106">
@@ -2840,11 +2829,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F106" s="2">
-        <v>46174</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="107">
@@ -2860,11 +2849,14 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Julho</t>
-        </is>
+          <t>Março</t>
+        </is>
+      </c>
+      <c r="D107">
+        <v>671.45</v>
       </c>
       <c r="F107" s="2">
-        <v>46204</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="108">
@@ -2880,11 +2872,17 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="D108">
+        <v>702.71</v>
+      </c>
+      <c r="E108">
+        <v>4.66</v>
       </c>
       <c r="F108" s="2">
-        <v>46235</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="109">
@@ -2900,17 +2898,23 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Setembro</t>
-        </is>
+          <t>Maio</t>
+        </is>
+      </c>
+      <c r="D109">
+        <v>760.8099999999999</v>
+      </c>
+      <c r="E109">
+        <v>8.27</v>
       </c>
       <c r="F109" s="2">
-        <v>46266</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Indaial</t>
+          <t>Bombinhas</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -2920,17 +2924,17 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F110" s="2">
-        <v>46023</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Indaial</t>
+          <t>Bombinhas</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -2940,17 +2944,17 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F111" s="2">
-        <v>46054</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Indaial</t>
+          <t>Bombinhas</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -2960,17 +2964,17 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="F112" s="2">
-        <v>46082</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Indaial</t>
+          <t>Bombinhas</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -2980,20 +2984,17 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="D113">
-        <v>702.88</v>
+          <t>Setembro</t>
+        </is>
       </c>
       <c r="F113" s="2">
-        <v>46113</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Indaial</t>
+          <t>Bombinhas</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3003,11 +3004,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Outubro</t>
         </is>
       </c>
       <c r="F114" s="2">
-        <v>46143</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="115">
@@ -3023,11 +3024,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F115" s="2">
-        <v>46174</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="116">
@@ -3043,11 +3044,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F116" s="2">
-        <v>46204</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="117">
@@ -3063,14 +3064,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="D117">
-        <v>639.98</v>
+          <t>Março</t>
+        </is>
       </c>
       <c r="F117" s="2">
-        <v>46235</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="118">
@@ -3086,17 +3084,14 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="D118">
-        <v>690.5599999999999</v>
-      </c>
-      <c r="E118">
-        <v>7.9</v>
+        <v>702.88</v>
       </c>
       <c r="F118" s="2">
-        <v>46266</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="119">
@@ -3110,17 +3105,19 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="D119">
-        <v>678.16</v>
-      </c>
-      <c r="E119">
-        <v>-1.8</v>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Maio</t>
+        </is>
+      </c>
+      <c r="F119" s="2">
+        <v>46143</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Jaraguá do Sul</t>
+          <t>Indaial</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3130,17 +3127,17 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F120" s="2">
-        <v>46023</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Jaraguá do Sul</t>
+          <t>Indaial</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3150,17 +3147,17 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F121" s="2">
-        <v>46054</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Jaraguá do Sul</t>
+          <t>Indaial</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3170,20 +3167,20 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="D122">
-        <v>642.83</v>
+        <v>639.98</v>
       </c>
       <c r="F122" s="2">
-        <v>46082</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Jaraguá do Sul</t>
+          <t>Indaial</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3193,23 +3190,23 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="D123">
-        <v>723.75</v>
+        <v>690.5599999999999</v>
       </c>
       <c r="E123">
-        <v>12.59</v>
+        <v>7.9</v>
       </c>
       <c r="F123" s="2">
-        <v>46113</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Jaraguá do Sul</t>
+          <t>Indaial</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3219,17 +3216,23 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Maio</t>
-        </is>
+          <t>Outubro</t>
+        </is>
+      </c>
+      <c r="D124">
+        <v>735.7</v>
+      </c>
+      <c r="E124">
+        <v>6.54</v>
       </c>
       <c r="F124" s="2">
-        <v>46143</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Jaraguá do Sul</t>
+          <t>Indaial</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3237,13 +3240,11 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>Junho</t>
-        </is>
-      </c>
-      <c r="F125" s="2">
-        <v>46174</v>
+      <c r="D125">
+        <v>678.16</v>
+      </c>
+      <c r="E125">
+        <v>-7.82</v>
       </c>
     </row>
     <row r="126">
@@ -3259,11 +3260,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F126" s="2">
-        <v>46204</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="127">
@@ -3279,14 +3280,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="D127">
-        <v>623.02</v>
+          <t>Fevereiro</t>
+        </is>
       </c>
       <c r="F127" s="2">
-        <v>46235</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="128">
@@ -3302,23 +3300,20 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="D128">
-        <v>674.26</v>
-      </c>
-      <c r="E128">
-        <v>8.220000000000001</v>
+        <v>642.83</v>
       </c>
       <c r="F128" s="2">
-        <v>46266</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Massaranduba</t>
+          <t>Jaraguá do Sul</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3328,17 +3323,23 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Janeiro</t>
-        </is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="D129">
+        <v>723.75</v>
+      </c>
+      <c r="E129">
+        <v>12.59</v>
       </c>
       <c r="F129" s="2">
-        <v>46023</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Massaranduba</t>
+          <t>Jaraguá do Sul</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3348,17 +3349,17 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F130" s="2">
-        <v>46054</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Massaranduba</t>
+          <t>Jaraguá do Sul</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3368,17 +3369,17 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F131" s="2">
-        <v>46082</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Massaranduba</t>
+          <t>Jaraguá do Sul</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3388,20 +3389,17 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="D132">
-        <v>593.53</v>
+          <t>Julho</t>
+        </is>
       </c>
       <c r="F132" s="2">
-        <v>46113</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Massaranduba</t>
+          <t>Jaraguá do Sul</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3411,17 +3409,20 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Maio</t>
-        </is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="D133">
+        <v>623.02</v>
       </c>
       <c r="F133" s="2">
-        <v>46143</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Massaranduba</t>
+          <t>Jaraguá do Sul</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3431,17 +3432,23 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Junho</t>
-        </is>
+          <t>Setembro</t>
+        </is>
+      </c>
+      <c r="D134">
+        <v>674.26</v>
+      </c>
+      <c r="E134">
+        <v>8.220000000000001</v>
       </c>
       <c r="F134" s="2">
-        <v>46174</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Massaranduba</t>
+          <t>Jaraguá do Sul</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3451,11 +3458,17 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Julho</t>
-        </is>
+          <t>Outubro</t>
+        </is>
+      </c>
+      <c r="D135">
+        <v>738.79</v>
+      </c>
+      <c r="E135">
+        <v>9.57</v>
       </c>
       <c r="F135" s="2">
-        <v>46204</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="136">
@@ -3471,14 +3484,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="D136">
-        <v>653.8</v>
+          <t>Janeiro</t>
+        </is>
       </c>
       <c r="F136" s="2">
-        <v>46235</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="137">
@@ -3494,23 +3504,17 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Setembro</t>
-        </is>
-      </c>
-      <c r="D137">
-        <v>694.64</v>
-      </c>
-      <c r="E137">
-        <v>6.25</v>
+          <t>Fevereiro</t>
+        </is>
       </c>
       <c r="F137" s="2">
-        <v>46266</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Navegantes</t>
+          <t>Massaranduba</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3520,17 +3524,17 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="F138" s="2">
-        <v>46023</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Navegantes</t>
+          <t>Massaranduba</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -3540,17 +3544,20 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
-        </is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="D139">
+        <v>593.53</v>
       </c>
       <c r="F139" s="2">
-        <v>46054</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Navegantes</t>
+          <t>Massaranduba</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -3560,17 +3567,17 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F140" s="2">
-        <v>46082</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Navegantes</t>
+          <t>Massaranduba</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -3580,20 +3587,17 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="D141">
-        <v>684.72</v>
+          <t>Junho</t>
+        </is>
       </c>
       <c r="F141" s="2">
-        <v>46113</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Navegantes</t>
+          <t>Massaranduba</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3603,17 +3607,17 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F142" s="2">
-        <v>46143</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Navegantes</t>
+          <t>Massaranduba</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3623,17 +3627,20 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Junho</t>
-        </is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="D143">
+        <v>653.8</v>
       </c>
       <c r="F143" s="2">
-        <v>46174</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Navegantes</t>
+          <t>Massaranduba</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3643,17 +3650,23 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Julho</t>
-        </is>
+          <t>Setembro</t>
+        </is>
+      </c>
+      <c r="D144">
+        <v>694.64</v>
+      </c>
+      <c r="E144">
+        <v>6.25</v>
       </c>
       <c r="F144" s="2">
-        <v>46204</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Navegantes</t>
+          <t>Massaranduba</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3663,11 +3676,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Outubro</t>
         </is>
       </c>
       <c r="F145" s="2">
-        <v>46235</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="146">
@@ -3683,17 +3696,17 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F146" s="2">
-        <v>46266</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Timbó</t>
+          <t>Navegantes</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -3703,17 +3716,17 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F147" s="2">
-        <v>46023</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Timbó</t>
+          <t>Navegantes</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -3723,17 +3736,17 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="F148" s="2">
-        <v>46054</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Timbó</t>
+          <t>Navegantes</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -3743,17 +3756,20 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Março</t>
-        </is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="D149">
+        <v>684.72</v>
       </c>
       <c r="F149" s="2">
-        <v>46082</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Timbó</t>
+          <t>Navegantes</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -3763,20 +3779,17 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="D150">
-        <v>760.12</v>
+          <t>Maio</t>
+        </is>
       </c>
       <c r="F150" s="2">
-        <v>46113</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Timbó</t>
+          <t>Navegantes</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -3786,17 +3799,17 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F151" s="2">
-        <v>46143</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Timbó</t>
+          <t>Navegantes</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -3806,17 +3819,17 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F152" s="2">
-        <v>46174</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Timbó</t>
+          <t>Navegantes</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -3826,17 +3839,17 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="F153" s="2">
-        <v>46204</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Timbó</t>
+          <t>Navegantes</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -3846,20 +3859,17 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="D154">
-        <v>650.8200000000001</v>
+          <t>Setembro</t>
+        </is>
       </c>
       <c r="F154" s="2">
-        <v>46235</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Timbó</t>
+          <t>Navegantes</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -3869,23 +3879,17 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Setembro</t>
-        </is>
-      </c>
-      <c r="D155">
-        <v>641.26</v>
-      </c>
-      <c r="E155">
-        <v>-1.47</v>
+          <t>Outubro</t>
+        </is>
       </c>
       <c r="F155" s="2">
-        <v>46266</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Balneário Camboriú</t>
+          <t>Timbó</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -3905,7 +3909,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Balneário Camboriú</t>
+          <t>Timbó</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -3925,7 +3929,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Balneário Camboriú</t>
+          <t>Timbó</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -3945,7 +3949,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Balneário Camboriú</t>
+          <t>Timbó</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -3957,6 +3961,9 @@
         <is>
           <t>Abril</t>
         </is>
+      </c>
+      <c r="D159">
+        <v>760.12</v>
       </c>
       <c r="F159" s="2">
         <v>46113</v>
@@ -3965,7 +3972,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Balneário Camboriú</t>
+          <t>Timbó</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -3985,7 +3992,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Balneário Camboriú</t>
+          <t>Timbó</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4005,7 +4012,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Balneário Camboriú</t>
+          <t>Timbó</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4025,7 +4032,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Balneário Camboriú</t>
+          <t>Timbó</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4039,7 +4046,7 @@
         </is>
       </c>
       <c r="D163">
-        <v>689.67</v>
+        <v>650.8200000000001</v>
       </c>
       <c r="F163" s="2">
         <v>46235</v>
@@ -4048,7 +4055,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Balneário Camboriú</t>
+          <t>Timbó</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -4062,10 +4069,10 @@
         </is>
       </c>
       <c r="D164">
-        <v>738.25</v>
+        <v>641.26</v>
       </c>
       <c r="E164">
-        <v>7.04</v>
+        <v>-1.47</v>
       </c>
       <c r="F164" s="2">
         <v>46266</v>
@@ -4074,7 +4081,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Pomerode</t>
+          <t>Timbó</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -4084,17 +4091,23 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Janeiro</t>
-        </is>
+          <t>Outubro</t>
+        </is>
+      </c>
+      <c r="D165">
+        <v>708.75</v>
+      </c>
+      <c r="E165">
+        <v>10.52</v>
       </c>
       <c r="F165" s="2">
-        <v>46023</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Pomerode</t>
+          <t>Balneário Camboriú</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4104,17 +4117,17 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F166" s="2">
-        <v>46054</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Pomerode</t>
+          <t>Balneário Camboriú</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4124,17 +4137,17 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F167" s="2">
-        <v>46082</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Pomerode</t>
+          <t>Balneário Camboriú</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4144,17 +4157,17 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="F168" s="2">
-        <v>46113</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Pomerode</t>
+          <t>Balneário Camboriú</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -4164,17 +4177,17 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="F169" s="2">
-        <v>46143</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Pomerode</t>
+          <t>Balneário Camboriú</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4184,17 +4197,17 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F170" s="2">
-        <v>46174</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Pomerode</t>
+          <t>Balneário Camboriú</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4204,17 +4217,17 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F171" s="2">
-        <v>46204</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Pomerode</t>
+          <t>Balneário Camboriú</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4224,40 +4237,313 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="D172">
-        <v>705.25</v>
+          <t>Julho</t>
+        </is>
       </c>
       <c r="F172" s="2">
-        <v>46235</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
+          <t>Balneário Camboriú</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="D173">
+        <v>689.67</v>
+      </c>
+      <c r="F173" s="2">
+        <v>46235</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Balneário Camboriú</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Setembro</t>
+        </is>
+      </c>
+      <c r="D174">
+        <v>738.25</v>
+      </c>
+      <c r="E174">
+        <v>7.04</v>
+      </c>
+      <c r="F174" s="2">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Balneário Camboriú</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Outubro</t>
+        </is>
+      </c>
+      <c r="D175">
+        <v>772.09</v>
+      </c>
+      <c r="E175">
+        <v>4.58</v>
+      </c>
+      <c r="F175" s="2">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Balneário Camboriú</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D176">
+        <v>788.86</v>
+      </c>
+      <c r="E176">
+        <v>2.17</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
           <t>Pomerode</t>
         </is>
       </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Janeiro</t>
+        </is>
+      </c>
+      <c r="F177" s="2">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Fevereiro</t>
+        </is>
+      </c>
+      <c r="F178" s="2">
+        <v>46054</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Março</t>
+        </is>
+      </c>
+      <c r="F179" s="2">
+        <v>46082</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="F180" s="2">
+        <v>46113</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Maio</t>
+        </is>
+      </c>
+      <c r="F181" s="2">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Junho</t>
+        </is>
+      </c>
+      <c r="F182" s="2">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Julho</t>
+        </is>
+      </c>
+      <c r="F183" s="2">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Agosto</t>
+        </is>
+      </c>
+      <c r="D184">
+        <v>705.25</v>
+      </c>
+      <c r="F184" s="2">
+        <v>46235</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
         <is>
           <t>Setembro</t>
         </is>
       </c>
-      <c r="D173">
+      <c r="D185">
         <v>751.7</v>
       </c>
-      <c r="E173">
+      <c r="E185">
         <v>6.59</v>
       </c>
-      <c r="F173" s="2">
+      <c r="F185" s="2">
         <v>46266</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Outubro</t>
+        </is>
+      </c>
+      <c r="F186" s="2">
+        <v>46296</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add October 2026 market data
Add October 2026 supermarket price files and refresh the compiled RDS/XLSX datasets and Shiny deployment metadata.
</commit_message>
<xml_diff>
--- a/CT.xlsx
+++ b/CT.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F186"/>
+  <dimension ref="A1:F187"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="6" max="6" width="20.7109375" style="2" customWidth="1"/>
@@ -1519,6 +1519,12 @@
           <t>Outubro</t>
         </is>
       </c>
+      <c r="D47">
+        <v>723</v>
+      </c>
+      <c r="E47">
+        <v>6.45</v>
+      </c>
       <c r="F47" s="2">
         <v>46296</v>
       </c>
@@ -2304,6 +2310,12 @@
           <t>Outubro</t>
         </is>
       </c>
+      <c r="D81">
+        <v>681.54</v>
+      </c>
+      <c r="E81">
+        <v>9.06</v>
+      </c>
       <c r="F81" s="2">
         <v>46296</v>
       </c>
@@ -2311,21 +2323,19 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Brusque</t>
+          <t>Gaspar</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>Janeiro</t>
-        </is>
-      </c>
-      <c r="F82" s="2">
-        <v>45658</v>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D82">
+        <v>604.4400000000001</v>
+      </c>
+      <c r="E82">
+        <v>-11.31</v>
       </c>
     </row>
     <row r="83">
@@ -2341,11 +2351,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F83" s="2">
-        <v>45689</v>
+        <v>45658</v>
       </c>
     </row>
     <row r="84">
@@ -2361,11 +2371,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F84" s="2">
-        <v>45717</v>
+        <v>45689</v>
       </c>
     </row>
     <row r="85">
@@ -2381,11 +2391,11 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="F85" s="2">
-        <v>45748</v>
+        <v>45717</v>
       </c>
     </row>
     <row r="86">
@@ -2401,11 +2411,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="F86" s="2">
-        <v>45778</v>
+        <v>45748</v>
       </c>
     </row>
     <row r="87">
@@ -2421,11 +2431,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F87" s="2">
-        <v>45809</v>
+        <v>45778</v>
       </c>
     </row>
     <row r="88">
@@ -2441,11 +2451,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F88" s="2">
-        <v>45839</v>
+        <v>45809</v>
       </c>
     </row>
     <row r="89">
@@ -2461,11 +2471,11 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F89" s="2">
-        <v>45870</v>
+        <v>45839</v>
       </c>
     </row>
     <row r="90">
@@ -2481,14 +2491,11 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Setembro</t>
-        </is>
-      </c>
-      <c r="D90">
-        <v>632.52</v>
+          <t>Agosto</t>
+        </is>
       </c>
       <c r="F90" s="2">
-        <v>45901</v>
+        <v>45870</v>
       </c>
     </row>
     <row r="91">
@@ -2504,17 +2511,14 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Outubro</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="D91">
-        <v>648.67</v>
-      </c>
-      <c r="E91">
-        <v>2.55</v>
+        <v>632.52</v>
       </c>
       <c r="F91" s="2">
-        <v>45931</v>
+        <v>45901</v>
       </c>
     </row>
     <row r="92">
@@ -2530,17 +2534,17 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Novembro</t>
+          <t>Outubro</t>
         </is>
       </c>
       <c r="D92">
-        <v>625.33</v>
+        <v>648.67</v>
       </c>
       <c r="E92">
-        <v>-3.6</v>
+        <v>2.55</v>
       </c>
       <c r="F92" s="2">
-        <v>45962</v>
+        <v>45931</v>
       </c>
     </row>
     <row r="93">
@@ -2556,11 +2560,17 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Dezembro</t>
-        </is>
+          <t>Novembro</t>
+        </is>
+      </c>
+      <c r="D93">
+        <v>625.33</v>
+      </c>
+      <c r="E93">
+        <v>-3.6</v>
       </c>
       <c r="F93" s="2">
-        <v>45992</v>
+        <v>45962</v>
       </c>
     </row>
     <row r="94">
@@ -2571,16 +2581,16 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Dezembro</t>
         </is>
       </c>
       <c r="F94" s="2">
-        <v>46023</v>
+        <v>45992</v>
       </c>
     </row>
     <row r="95">
@@ -2596,11 +2606,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F95" s="2">
-        <v>46054</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="96">
@@ -2616,11 +2626,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F96" s="2">
-        <v>46082</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="97">
@@ -2636,11 +2646,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="F97" s="2">
-        <v>46113</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="98">
@@ -2656,11 +2666,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="F98" s="2">
-        <v>46143</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="99">
@@ -2676,11 +2686,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F99" s="2">
-        <v>46174</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="100">
@@ -2696,11 +2706,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F100" s="2">
-        <v>46204</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="101">
@@ -2716,14 +2726,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="D101">
-        <v>700.12</v>
+          <t>Julho</t>
+        </is>
       </c>
       <c r="F101" s="2">
-        <v>46235</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="102">
@@ -2739,17 +2746,14 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="D102">
-        <v>697.37</v>
-      </c>
-      <c r="E102">
-        <v>-0.39</v>
+        <v>700.12</v>
       </c>
       <c r="F102" s="2">
-        <v>46266</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="103">
@@ -2765,17 +2769,17 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Outubro</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="D103">
-        <v>762.29</v>
+        <v>697.37</v>
       </c>
       <c r="E103">
-        <v>9.31</v>
+        <v>-0.39</v>
       </c>
       <c r="F103" s="2">
-        <v>46296</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="104">
@@ -2789,17 +2793,25 @@
           <t>2026</t>
         </is>
       </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Outubro</t>
+        </is>
+      </c>
       <c r="D104">
-        <v>682.34</v>
+        <v>779.77</v>
       </c>
       <c r="E104">
-        <v>-10.49</v>
+        <v>11.82</v>
+      </c>
+      <c r="F104" s="2">
+        <v>46296</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Bombinhas</t>
+          <t>Brusque</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2807,13 +2819,11 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>Janeiro</t>
-        </is>
-      </c>
-      <c r="F105" s="2">
-        <v>46023</v>
+      <c r="D105">
+        <v>682.34</v>
+      </c>
+      <c r="E105">
+        <v>-12.49</v>
       </c>
     </row>
     <row r="106">
@@ -2829,11 +2839,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F106" s="2">
-        <v>46054</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="107">
@@ -2849,14 +2859,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Março</t>
-        </is>
-      </c>
-      <c r="D107">
-        <v>671.45</v>
+          <t>Fevereiro</t>
+        </is>
       </c>
       <c r="F107" s="2">
-        <v>46082</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="108">
@@ -2872,17 +2879,14 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="D108">
-        <v>702.71</v>
-      </c>
-      <c r="E108">
-        <v>4.66</v>
+        <v>671.45</v>
       </c>
       <c r="F108" s="2">
-        <v>46113</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="109">
@@ -2898,17 +2902,17 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="D109">
-        <v>760.8099999999999</v>
+        <v>702.71</v>
       </c>
       <c r="E109">
-        <v>8.27</v>
+        <v>4.66</v>
       </c>
       <c r="F109" s="2">
-        <v>46143</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="110">
@@ -2924,11 +2928,17 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Junho</t>
-        </is>
+          <t>Maio</t>
+        </is>
+      </c>
+      <c r="D110">
+        <v>760.8099999999999</v>
+      </c>
+      <c r="E110">
+        <v>8.27</v>
       </c>
       <c r="F110" s="2">
-        <v>46174</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="111">
@@ -2944,11 +2954,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F111" s="2">
-        <v>46204</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="112">
@@ -2964,11 +2974,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F112" s="2">
-        <v>46235</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="113">
@@ -2984,11 +2994,11 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="F113" s="2">
-        <v>46266</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="114">
@@ -3004,17 +3014,17 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Outubro</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="F114" s="2">
-        <v>46296</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Indaial</t>
+          <t>Bombinhas</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3024,11 +3034,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Outubro</t>
         </is>
       </c>
       <c r="F115" s="2">
-        <v>46023</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="116">
@@ -3044,11 +3054,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F116" s="2">
-        <v>46054</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="117">
@@ -3064,11 +3074,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F117" s="2">
-        <v>46082</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="118">
@@ -3084,14 +3094,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="D118">
-        <v>702.88</v>
+          <t>Março</t>
+        </is>
       </c>
       <c r="F118" s="2">
-        <v>46113</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="119">
@@ -3107,11 +3114,14 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Maio</t>
-        </is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="D119">
+        <v>702.88</v>
       </c>
       <c r="F119" s="2">
-        <v>46143</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="120">
@@ -3127,11 +3137,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F120" s="2">
-        <v>46174</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="121">
@@ -3147,11 +3157,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F121" s="2">
-        <v>46204</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="122">
@@ -3167,14 +3177,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="D122">
-        <v>639.98</v>
+          <t>Julho</t>
+        </is>
       </c>
       <c r="F122" s="2">
-        <v>46235</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="123">
@@ -3190,17 +3197,14 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="D123">
-        <v>690.5599999999999</v>
-      </c>
-      <c r="E123">
-        <v>7.9</v>
+        <v>639.98</v>
       </c>
       <c r="F123" s="2">
-        <v>46266</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="124">
@@ -3216,17 +3220,17 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Outubro</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="D124">
-        <v>735.7</v>
+        <v>690.5599999999999</v>
       </c>
       <c r="E124">
-        <v>6.54</v>
+        <v>7.9</v>
       </c>
       <c r="F124" s="2">
-        <v>46296</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="125">
@@ -3240,17 +3244,25 @@
           <t>2026</t>
         </is>
       </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Outubro</t>
+        </is>
+      </c>
       <c r="D125">
-        <v>678.16</v>
+        <v>735.7</v>
       </c>
       <c r="E125">
-        <v>-7.82</v>
+        <v>6.54</v>
+      </c>
+      <c r="F125" s="2">
+        <v>46296</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Jaraguá do Sul</t>
+          <t>Indaial</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3258,13 +3270,11 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>Janeiro</t>
-        </is>
-      </c>
-      <c r="F126" s="2">
-        <v>46023</v>
+      <c r="D126">
+        <v>678.16</v>
+      </c>
+      <c r="E126">
+        <v>-7.82</v>
       </c>
     </row>
     <row r="127">
@@ -3280,11 +3290,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F127" s="2">
-        <v>46054</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="128">
@@ -3300,14 +3310,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Março</t>
-        </is>
-      </c>
-      <c r="D128">
-        <v>642.83</v>
+          <t>Fevereiro</t>
+        </is>
       </c>
       <c r="F128" s="2">
-        <v>46082</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="129">
@@ -3323,17 +3330,14 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="D129">
-        <v>723.75</v>
-      </c>
-      <c r="E129">
-        <v>12.59</v>
+        <v>642.83</v>
       </c>
       <c r="F129" s="2">
-        <v>46113</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="130">
@@ -3349,11 +3353,17 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Maio</t>
-        </is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="D130">
+        <v>723.75</v>
+      </c>
+      <c r="E130">
+        <v>12.59</v>
       </c>
       <c r="F130" s="2">
-        <v>46143</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="131">
@@ -3369,11 +3379,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F131" s="2">
-        <v>46174</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="132">
@@ -3389,11 +3399,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F132" s="2">
-        <v>46204</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="133">
@@ -3409,14 +3419,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="D133">
-        <v>623.02</v>
+          <t>Julho</t>
+        </is>
       </c>
       <c r="F133" s="2">
-        <v>46235</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="134">
@@ -3432,17 +3439,14 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="D134">
-        <v>674.26</v>
-      </c>
-      <c r="E134">
-        <v>8.220000000000001</v>
+        <v>623.02</v>
       </c>
       <c r="F134" s="2">
-        <v>46266</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="135">
@@ -3458,23 +3462,23 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Outubro</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="D135">
-        <v>738.79</v>
+        <v>674.26</v>
       </c>
       <c r="E135">
-        <v>9.57</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="F135" s="2">
-        <v>46296</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Massaranduba</t>
+          <t>Jaraguá do Sul</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3484,11 +3488,17 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Janeiro</t>
-        </is>
+          <t>Outubro</t>
+        </is>
+      </c>
+      <c r="D136">
+        <v>738.79</v>
+      </c>
+      <c r="E136">
+        <v>9.57</v>
       </c>
       <c r="F136" s="2">
-        <v>46023</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="137">
@@ -3504,11 +3514,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F137" s="2">
-        <v>46054</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="138">
@@ -3524,11 +3534,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F138" s="2">
-        <v>46082</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="139">
@@ -3544,14 +3554,11 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="D139">
-        <v>593.53</v>
+          <t>Março</t>
+        </is>
       </c>
       <c r="F139" s="2">
-        <v>46113</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="140">
@@ -3567,11 +3574,14 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Maio</t>
-        </is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="D140">
+        <v>593.53</v>
       </c>
       <c r="F140" s="2">
-        <v>46143</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="141">
@@ -3587,11 +3597,11 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F141" s="2">
-        <v>46174</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="142">
@@ -3607,11 +3617,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F142" s="2">
-        <v>46204</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="143">
@@ -3627,14 +3637,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="D143">
-        <v>653.8</v>
+          <t>Julho</t>
+        </is>
       </c>
       <c r="F143" s="2">
-        <v>46235</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="144">
@@ -3650,17 +3657,14 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="D144">
-        <v>694.64</v>
-      </c>
-      <c r="E144">
-        <v>6.25</v>
+        <v>653.8</v>
       </c>
       <c r="F144" s="2">
-        <v>46266</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="145">
@@ -3676,17 +3680,23 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Outubro</t>
-        </is>
+          <t>Setembro</t>
+        </is>
+      </c>
+      <c r="D145">
+        <v>694.64</v>
+      </c>
+      <c r="E145">
+        <v>6.25</v>
       </c>
       <c r="F145" s="2">
-        <v>46296</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Navegantes</t>
+          <t>Massaranduba</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3696,11 +3706,17 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Janeiro</t>
-        </is>
+          <t>Outubro</t>
+        </is>
+      </c>
+      <c r="D146">
+        <v>723.79</v>
+      </c>
+      <c r="E146">
+        <v>4.2</v>
       </c>
       <c r="F146" s="2">
-        <v>46023</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="147">
@@ -3716,11 +3732,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F147" s="2">
-        <v>46054</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="148">
@@ -3736,11 +3752,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F148" s="2">
-        <v>46082</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="149">
@@ -3756,14 +3772,11 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="D149">
-        <v>684.72</v>
+          <t>Março</t>
+        </is>
       </c>
       <c r="F149" s="2">
-        <v>46113</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="150">
@@ -3779,11 +3792,14 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Maio</t>
-        </is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="D150">
+        <v>684.72</v>
       </c>
       <c r="F150" s="2">
-        <v>46143</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="151">
@@ -3799,11 +3815,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F151" s="2">
-        <v>46174</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="152">
@@ -3819,11 +3835,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F152" s="2">
-        <v>46204</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="153">
@@ -3839,11 +3855,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="F153" s="2">
-        <v>46235</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="154">
@@ -3859,11 +3875,11 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="F154" s="2">
-        <v>46266</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="155">
@@ -3879,17 +3895,17 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Outubro</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="F155" s="2">
-        <v>46296</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Timbó</t>
+          <t>Navegantes</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -3899,11 +3915,11 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>Outubro</t>
         </is>
       </c>
       <c r="F156" s="2">
-        <v>46023</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="157">
@@ -3919,11 +3935,11 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F157" s="2">
-        <v>46054</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="158">
@@ -3939,11 +3955,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F158" s="2">
-        <v>46082</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="159">
@@ -3959,14 +3975,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="D159">
-        <v>760.12</v>
+          <t>Março</t>
+        </is>
       </c>
       <c r="F159" s="2">
-        <v>46113</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="160">
@@ -3982,11 +3995,14 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Maio</t>
-        </is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="D160">
+        <v>760.12</v>
       </c>
       <c r="F160" s="2">
-        <v>46143</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="161">
@@ -4002,11 +4018,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F161" s="2">
-        <v>46174</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="162">
@@ -4022,11 +4038,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F162" s="2">
-        <v>46204</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="163">
@@ -4042,14 +4058,11 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="D163">
-        <v>650.8200000000001</v>
+          <t>Julho</t>
+        </is>
       </c>
       <c r="F163" s="2">
-        <v>46235</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="164">
@@ -4065,17 +4078,14 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="D164">
-        <v>641.26</v>
-      </c>
-      <c r="E164">
-        <v>-1.47</v>
+        <v>650.8200000000001</v>
       </c>
       <c r="F164" s="2">
-        <v>46266</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="165">
@@ -4091,23 +4101,23 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Outubro</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="D165">
-        <v>708.75</v>
+        <v>641.26</v>
       </c>
       <c r="E165">
-        <v>10.52</v>
+        <v>-1.47</v>
       </c>
       <c r="F165" s="2">
-        <v>46296</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Balneário Camboriú</t>
+          <t>Timbó</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4117,11 +4127,17 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Janeiro</t>
-        </is>
+          <t>Outubro</t>
+        </is>
+      </c>
+      <c r="D166">
+        <v>708.75</v>
+      </c>
+      <c r="E166">
+        <v>10.52</v>
       </c>
       <c r="F166" s="2">
-        <v>46023</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="167">
@@ -4137,11 +4153,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F167" s="2">
-        <v>46054</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="168">
@@ -4157,11 +4173,11 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F168" s="2">
-        <v>46082</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="169">
@@ -4177,11 +4193,11 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="F169" s="2">
-        <v>46113</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="170">
@@ -4197,11 +4213,11 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="F170" s="2">
-        <v>46143</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="171">
@@ -4217,11 +4233,11 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F171" s="2">
-        <v>46174</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="172">
@@ -4237,11 +4253,11 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F172" s="2">
-        <v>46204</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="173">
@@ -4257,14 +4273,11 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="D173">
-        <v>689.67</v>
+          <t>Julho</t>
+        </is>
       </c>
       <c r="F173" s="2">
-        <v>46235</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="174">
@@ -4280,17 +4293,14 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="D174">
-        <v>738.25</v>
-      </c>
-      <c r="E174">
-        <v>7.04</v>
+        <v>689.67</v>
       </c>
       <c r="F174" s="2">
-        <v>46266</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="175">
@@ -4306,17 +4316,17 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Outubro</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="D175">
-        <v>772.09</v>
+        <v>738.25</v>
       </c>
       <c r="E175">
-        <v>4.58</v>
+        <v>7.04</v>
       </c>
       <c r="F175" s="2">
-        <v>46296</v>
+        <v>46266</v>
       </c>
     </row>
     <row r="176">
@@ -4330,17 +4340,25 @@
           <t>2026</t>
         </is>
       </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Outubro</t>
+        </is>
+      </c>
       <c r="D176">
-        <v>788.86</v>
+        <v>772.09</v>
       </c>
       <c r="E176">
-        <v>2.17</v>
+        <v>4.58</v>
+      </c>
+      <c r="F176" s="2">
+        <v>46296</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Pomerode</t>
+          <t>Balneário Camboriú</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -4348,13 +4366,11 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>Janeiro</t>
-        </is>
-      </c>
-      <c r="F177" s="2">
-        <v>46023</v>
+      <c r="D177">
+        <v>788.86</v>
+      </c>
+      <c r="E177">
+        <v>2.17</v>
       </c>
     </row>
     <row r="178">
@@ -4370,11 +4386,11 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>Janeiro</t>
         </is>
       </c>
       <c r="F178" s="2">
-        <v>46054</v>
+        <v>46023</v>
       </c>
     </row>
     <row r="179">
@@ -4390,11 +4406,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="F179" s="2">
-        <v>46082</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="180">
@@ -4410,11 +4426,11 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="F180" s="2">
-        <v>46113</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="181">
@@ -4430,11 +4446,11 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="F181" s="2">
-        <v>46143</v>
+        <v>46113</v>
       </c>
     </row>
     <row r="182">
@@ -4450,11 +4466,11 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="F182" s="2">
-        <v>46174</v>
+        <v>46143</v>
       </c>
     </row>
     <row r="183">
@@ -4470,11 +4486,11 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="F183" s="2">
-        <v>46204</v>
+        <v>46174</v>
       </c>
     </row>
     <row r="184">
@@ -4490,14 +4506,11 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="D184">
-        <v>705.25</v>
+          <t>Julho</t>
+        </is>
       </c>
       <c r="F184" s="2">
-        <v>46235</v>
+        <v>46204</v>
       </c>
     </row>
     <row r="185">
@@ -4513,17 +4526,14 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="D185">
-        <v>751.7</v>
-      </c>
-      <c r="E185">
-        <v>6.59</v>
+        <v>705.25</v>
       </c>
       <c r="F185" s="2">
-        <v>46266</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="186">
@@ -4539,10 +4549,36 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
+          <t>Setembro</t>
+        </is>
+      </c>
+      <c r="D186">
+        <v>751.7</v>
+      </c>
+      <c r="E186">
+        <v>6.59</v>
+      </c>
+      <c r="F186" s="2">
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Pomerode</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
           <t>Outubro</t>
         </is>
       </c>
-      <c r="F186" s="2">
+      <c r="F187" s="2">
         <v>46296</v>
       </c>
     </row>

</xml_diff>